<commit_message>
Add noise/sound exposure assessment for all buildings
Added 'Noise exposure' (Low/Moderate/Elevated/High) and 'Noise notes'
columns rating outside-noise exposure for every building, driven by:
- Columbia's Frat Row (W 113th/114th, Broadway-Amsterdam) party noise
- arterials/transit: Broadway, W 125th + elevated 1 train, Henry Hudson Pkwy
- quiet streets: Riverside Dr, Claremont Ave, west-of-Broadway blocks

Each address was geocoded (US Census) to verify its east/west position
relative to Broadway. Methodology and caveats documented in the Read me.
</commit_message>
<xml_diff>
--- a/Columbia_CBS_Rentable_Amenities.xlsx
+++ b/Columbia_CBS_Rentable_Amenities.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -82,6 +82,9 @@
       <color rgb="00666666"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -137,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -181,6 +184,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -546,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -649,6 +653,125 @@
       <c r="A17" s="6" t="inlineStr">
         <is>
           <t>'Window' AC = resident purchases &amp; professionally installs a unit (CR default). '*Standard' = pre-war building where window AC is universal but the specific profile line wasn't separately re-confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>NOISE / SOUND EXPOSURE (new columns 'Noise exposure' + 'Noise notes'):</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Every building rated Low / Moderate / Elevated / High for likely outside-noise exposure. This is a LOCATION-BASED</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   assessment (street type + proximity to noise sources), not a per-unit interior measurement or a per-building review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Key drivers used:</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     • Frat Row = W 113th &amp; W 114th between Broadway and Amsterdam, with active Greek houses at ~534/536/540/548 W 114th</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       and 548/556 W 113th. Buildings on the 530–560 core = High (documented weekend/late-night party noise); the</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       Amsterdam-end (500–529) = Elevated. Columbia housing reviews describe this block as 'loud at night.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     • Major arterials/transit = High: Broadway (buses/traffic/bars), W 125th + the elevated 1-train viaduct (122nd–135th),</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       and the Henry Hudson Parkway (highway).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     • Quiet (Low): Riverside Drive, Claremont Ave, and the west-of-Broadway ends of the side streets (600+ numbers),</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       plus the calm faculty-housing blocks north of campus (116th–122nd).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     • Moderate: side streets one block off Frat Row (112th), near Broadway bar corners (111th, The Heights), campus-edge</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       blocks (115th near Butler), Morningside Drive (park-facing), and 74 W 108th.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Mitigation note: the central-air buildings (Broadway, 125th, Riverside, Henry Hudson) let you keep windows shut, which</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   meaningfully reduces perceived street noise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Honesty note: I could not find building-specific Reddit threads for most addresses; ratings are inferred from location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   East/west-of-Broadway position was verified by geocoding each address (US Census geocoder).</t>
         </is>
       </c>
     </row>
@@ -663,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:N101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -678,6 +801,8 @@
     <col width="50" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="70" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -741,6 +866,16 @@
           <t>Profile URL</t>
         </is>
       </c>
+      <c r="M1" s="15" t="inlineStr">
+        <is>
+          <t>Noise exposure</t>
+        </is>
+      </c>
+      <c r="N1" s="15" t="inlineStr">
+        <is>
+          <t>Noise notes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
@@ -803,6 +938,16 @@
           <t>https://residential.columbia.edu/content/3260-henry-hudson-parkway</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Directly on the Henry Hudson Parkway — steady highway traffic noise day and night. Central AC lets you keep windows shut, which blunts it.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -861,6 +1006,16 @@
           <t>https://residential.columbia.edu/content/542-west-112th-street</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Residential block one street south of Frat Row (113th); some weekend spillover, plus bar noise near the Broadway corner (The Heights, E's Bar around 112th–113th &amp; Broadway).</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -919,6 +1074,16 @@
           <t>https://residential.columbia.edu/content/560-riverside-drive</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Park/parkway-facing Riverside Drive — among the quietest CR locations; only modest Riverside Dr through-traffic. Central AC lets you keep windows shut, which blunts it.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -977,6 +1142,16 @@
           <t>https://residential.columbia.edu/content/600-west-125th-street</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Busy W 125th St corridor with the elevated 1-train viaduct (122nd–135th) a block east at Broadway/125th — both significant noise sources. Central AC lets you keep windows shut, which blunts it.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -1035,6 +1210,16 @@
           <t>https://residential.columbia.edu/content/130-morningside-drive</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Faces Morningside Park; residential and generally calm at night, but Morningside Dr carries some through-traffic.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -1093,6 +1278,16 @@
           <t>https://residential.columbia.edu/content/423-west-120th-street</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -1153,6 +1348,16 @@
           <t>https://residential.columbia.edu/content/524-west-114th-street</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Eastern (Amsterdam) end of the Frat Row block — party-noise spillover from the 530–556 houses plus Amsterdam Ave bar/foot traffic; less intense than the core.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -1211,6 +1416,16 @@
           <t>https://residential.columbia.edu/content/530-west-113th-street</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>On Columbia's Frat Row (W 113th–114th between Broadway and Amsterdam) amid active Greek houses (e.g. 534/536/540/548 W 114th, 556 W 113th). Expect weekend and late-night party noise — Columbia housing reviews flag this block as 'loud at night.'</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -1271,6 +1486,16 @@
           <t>https://residential.columbia.edu/content/600-west-114th-street</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Quiet, west-of-Broadway end of W 114th toward Riverside — away from the fraternity houses on the Broadway–Amsterdam stretch.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -1329,6 +1554,16 @@
           <t>https://residential.columbia.edu/content/601-west-115th-street</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>West-of-Broadway end of W 115th toward Riverside — quiet residential.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -1387,6 +1622,16 @@
           <t>https://residential.columbia.edu/content/100-morningside-drive</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Faces Morningside Park; residential and generally calm at night, but Morningside Dr carries some through-traffic.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -1445,6 +1690,16 @@
           <t>https://residential.columbia.edu/content/110-morningside-drive</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Faces Morningside Park; residential and generally calm at night, but Morningside Dr carries some through-traffic.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -1503,6 +1758,16 @@
           <t>https://residential.columbia.edu/content/124-la-salle-street</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Manhattanville block close to W 125th St and the elevated 1 train; some through-traffic, though the side street itself is calmer than 125th.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -1561,6 +1826,16 @@
           <t>https://residential.columbia.edu/content/150-claremont-avenue</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Quiet residential side street west of Broadway; little nightlife or through-traffic.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -1619,6 +1894,16 @@
           <t>https://residential.columbia.edu/content/181-claremont-avenue</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Quiet residential side street west of Broadway; little nightlife or through-traffic.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -1677,6 +1962,16 @@
           <t>https://residential.columbia.edu/content/195-claremont-avenue</t>
         </is>
       </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Quiet residential side street west of Broadway; little nightlife or through-traffic.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -1735,6 +2030,16 @@
           <t>https://residential.columbia.edu/content/2700-broadway</t>
         </is>
       </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>On Broadway, a major arterial: buses, traffic, sirens and late-night bar/restaurant noise. Central AC lets you keep windows shut, which blunts it.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -1793,6 +2098,16 @@
           <t>https://residential.columbia.edu/content/400-west-119th-street</t>
         </is>
       </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -1851,6 +2166,16 @@
           <t>https://residential.columbia.edu/content/401-west-118th-street</t>
         </is>
       </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
@@ -1909,6 +2234,16 @@
           <t>https://residential.columbia.edu/content/403-west-115th-street</t>
         </is>
       </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Campus-edge block near Amsterdam/Butler Library; student foot traffic by day, limited nightlife. One block north of Frat Row, so some weekend spillover.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -1967,6 +2302,16 @@
           <t>https://residential.columbia.edu/content/405-west-118th-street</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
@@ -2025,6 +2370,16 @@
           <t>https://residential.columbia.edu/content/411-west-115th-street</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Campus-edge block near Amsterdam/Butler Library; student foot traffic by day, limited nightlife. One block north of Frat Row, so some weekend spillover.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -2083,6 +2438,16 @@
           <t>https://residential.columbia.edu/content/414-west-120th-street</t>
         </is>
       </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
@@ -2141,6 +2506,16 @@
           <t>https://residential.columbia.edu/content/415-west-115th-street</t>
         </is>
       </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Campus-edge block near Amsterdam/Butler Library; student foot traffic by day, limited nightlife. One block north of Frat Row, so some weekend spillover.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -2199,6 +2574,16 @@
           <t>https://residential.columbia.edu/content/415-west-118th-street</t>
         </is>
       </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
@@ -2257,6 +2642,16 @@
           <t>https://residential.columbia.edu/content/417-west-118th-street</t>
         </is>
       </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
@@ -2315,6 +2710,16 @@
           <t>https://residential.columbia.edu/content/419-west-115th-street</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Campus-edge block near Amsterdam/Butler Library; student foot traffic by day, limited nightlife. One block north of Frat Row, so some weekend spillover.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
@@ -2373,6 +2778,16 @@
           <t>https://residential.columbia.edu/content/419-west-118th-street</t>
         </is>
       </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
@@ -2431,6 +2846,16 @@
           <t>https://residential.columbia.edu/content/419-west-119th-street</t>
         </is>
       </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
@@ -2489,6 +2914,16 @@
           <t>https://residential.columbia.edu/content/420-west-116th-street</t>
         </is>
       </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
@@ -2547,6 +2982,16 @@
           <t>https://residential.columbia.edu/content/420-west-119th-street</t>
         </is>
       </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
@@ -2605,6 +3050,16 @@
           <t>https://residential.columbia.edu/content/421-west-118th-street</t>
         </is>
       </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
@@ -2663,6 +3118,16 @@
           <t>https://residential.columbia.edu/content/423-west-118th-street</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
@@ -2721,6 +3186,16 @@
           <t>https://residential.columbia.edu/content/424-west-119th-street</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
@@ -2779,6 +3254,16 @@
           <t>https://residential.columbia.edu/content/434-west-120th-street</t>
         </is>
       </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
@@ -2837,6 +3322,16 @@
           <t>https://residential.columbia.edu/content/435-west-119th-street</t>
         </is>
       </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
@@ -2895,6 +3390,16 @@
           <t>https://residential.columbia.edu/content/500-west-122nd-street</t>
         </is>
       </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
@@ -2953,6 +3458,16 @@
           <t>https://residential.columbia.edu/content/501-west-121st-street</t>
         </is>
       </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
@@ -3011,6 +3526,16 @@
           <t>https://residential.columbia.edu/content/502-west-113th-street</t>
         </is>
       </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Eastern (Amsterdam) end of the Frat Row block — party-noise spillover from the 530–556 houses plus Amsterdam Ave bar/foot traffic; less intense than the core.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
@@ -3069,6 +3594,16 @@
           <t>https://residential.columbia.edu/content/502-west-122nd-street</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
@@ -3127,6 +3662,16 @@
           <t>https://residential.columbia.edu/content/506-west-113th-street</t>
         </is>
       </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Eastern (Amsterdam) end of the Frat Row block — party-noise spillover from the 530–556 houses plus Amsterdam Ave bar/foot traffic; less intense than the core.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
@@ -3185,6 +3730,16 @@
           <t>https://residential.columbia.edu/content/506-west-122nd-street</t>
         </is>
       </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
@@ -3243,6 +3798,16 @@
           <t>https://residential.columbia.edu/content/507-west-113th-street</t>
         </is>
       </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Eastern (Amsterdam) end of the Frat Row block — party-noise spillover from the 530–556 houses plus Amsterdam Ave bar/foot traffic; less intense than the core.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
@@ -3301,6 +3866,16 @@
           <t>https://residential.columbia.edu/content/509-west-112th-street</t>
         </is>
       </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>West-of-Broadway end of W 112th; quiet residential, away from the frat blocks.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
@@ -3359,6 +3934,16 @@
           <t>https://residential.columbia.edu/content/511-west-112th-street</t>
         </is>
       </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Residential block one street south of Frat Row (113th); some weekend spillover, plus bar noise near the Broadway corner (The Heights, E's Bar around 112th–113th &amp; Broadway).</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
@@ -3417,6 +4002,16 @@
           <t>https://residential.columbia.edu/content/511-west-113th-street</t>
         </is>
       </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Eastern (Amsterdam) end of the Frat Row block — party-noise spillover from the 530–556 houses plus Amsterdam Ave bar/foot traffic; less intense than the core.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
@@ -3475,6 +4070,16 @@
           <t>https://residential.columbia.edu/content/512-west-112th-street</t>
         </is>
       </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Residential block one street south of Frat Row (113th); some weekend spillover, plus bar noise near the Broadway corner (The Heights, E's Bar around 112th–113th &amp; Broadway).</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
@@ -3533,6 +4138,16 @@
           <t>https://residential.columbia.edu/content/514-west-114th-street</t>
         </is>
       </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Eastern (Amsterdam) end of the Frat Row block — party-noise spillover from the 530–556 houses plus Amsterdam Ave bar/foot traffic; less intense than the core.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
@@ -3591,6 +4206,16 @@
           <t>https://residential.columbia.edu/content/519-west-121st-street</t>
         </is>
       </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
@@ -3649,6 +4274,16 @@
           <t>https://residential.columbia.edu/content/520-west-114th-street</t>
         </is>
       </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Eastern (Amsterdam) end of the Frat Row block — party-noise spillover from the 530–556 houses plus Amsterdam Ave bar/foot traffic; less intense than the core.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
@@ -3707,6 +4342,16 @@
           <t>https://residential.columbia.edu/content/520-west-122nd-street</t>
         </is>
       </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
@@ -3765,6 +4410,16 @@
           <t>https://residential.columbia.edu/content/521-west-111th-street</t>
         </is>
       </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Residential block; main noise vectors are the Broadway corner (The Heights bar at 111th &amp; Broadway) and some weekend spillover from the 113th–114th frat blocks two streets north.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
@@ -3823,6 +4478,16 @@
           <t>https://residential.columbia.edu/content/521-west-112th-street</t>
         </is>
       </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Residential block one street south of Frat Row (113th); some weekend spillover, plus bar noise near the Broadway corner (The Heights, E's Bar around 112th–113th &amp; Broadway).</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
@@ -3881,6 +4546,16 @@
           <t>https://residential.columbia.edu/content/522-west-112th-street</t>
         </is>
       </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Residential block one street south of Frat Row (113th); some weekend spillover, plus bar noise near the Broadway corner (The Heights, E's Bar around 112th–113th &amp; Broadway).</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
@@ -3939,6 +4614,16 @@
           <t>https://residential.columbia.edu/content/523-west-112th-street</t>
         </is>
       </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Residential block one street south of Frat Row (113th); some weekend spillover, plus bar noise near the Broadway corner (The Heights, E's Bar around 112th–113th &amp; Broadway).</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
@@ -3997,6 +4682,16 @@
           <t>https://residential.columbia.edu/content/524-west-122nd-street</t>
         </is>
       </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
@@ -4055,6 +4750,16 @@
           <t>https://residential.columbia.edu/content/525-west-113th-street</t>
         </is>
       </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>Eastern (Amsterdam) end of the Frat Row block — party-noise spillover from the 530–556 houses plus Amsterdam Ave bar/foot traffic; less intense than the core.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
@@ -4113,6 +4818,16 @@
           <t>https://residential.columbia.edu/content/526-west-112th-street</t>
         </is>
       </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>Residential block one street south of Frat Row (113th); some weekend spillover, plus bar noise near the Broadway corner (The Heights, E's Bar around 112th–113th &amp; Broadway).</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
@@ -4171,6 +4886,16 @@
           <t>https://residential.columbia.edu/content/526-west-113th-street</t>
         </is>
       </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>Eastern (Amsterdam) end of the Frat Row block — party-noise spillover from the 530–556 houses plus Amsterdam Ave bar/foot traffic; less intense than the core.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
@@ -4229,6 +4954,16 @@
           <t>https://residential.columbia.edu/content/526-west-122nd-street</t>
         </is>
       </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
@@ -4287,6 +5022,16 @@
           <t>https://residential.columbia.edu/content/527-west-121st-street</t>
         </is>
       </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
@@ -4345,6 +5090,16 @@
           <t>https://residential.columbia.edu/content/528-riverside-drive</t>
         </is>
       </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>Park/parkway-facing Riverside Drive — among the quietest CR locations; only modest Riverside Dr through-traffic.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
@@ -4403,6 +5158,16 @@
           <t>https://residential.columbia.edu/content/528-west-114th-street</t>
         </is>
       </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>Eastern (Amsterdam) end of the Frat Row block — party-noise spillover from the 530–556 houses plus Amsterdam Ave bar/foot traffic; less intense than the core.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
@@ -4461,6 +5226,16 @@
           <t>https://residential.columbia.edu/content/529-west-111th-street</t>
         </is>
       </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>Residential block; main noise vectors are the Broadway corner (The Heights bar at 111th &amp; Broadway) and some weekend spillover from the 113th–114th frat blocks two streets north.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
@@ -4519,6 +5294,16 @@
           <t>https://residential.columbia.edu/content/530-riverside-drive</t>
         </is>
       </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>Park/parkway-facing Riverside Drive — among the quietest CR locations; only modest Riverside Dr through-traffic.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
@@ -4577,6 +5362,16 @@
           <t>https://residential.columbia.edu/content/530-west-112th-street</t>
         </is>
       </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>Residential block one street south of Frat Row (113th); some weekend spillover, plus bar noise near the Broadway corner (The Heights, E's Bar around 112th–113th &amp; Broadway).</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
@@ -4635,6 +5430,16 @@
           <t>https://residential.columbia.edu/content/530-west-114th-street</t>
         </is>
       </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>On Columbia's Frat Row (W 113th–114th between Broadway and Amsterdam) amid active Greek houses (e.g. 534/536/540/548 W 114th, 556 W 113th). Expect weekend and late-night party noise — Columbia housing reviews flag this block as 'loud at night.'</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
@@ -4693,6 +5498,16 @@
           <t>https://residential.columbia.edu/content/530-west-122nd-street</t>
         </is>
       </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
@@ -4751,6 +5566,16 @@
           <t>https://residential.columbia.edu/content/531-west-112th-street</t>
         </is>
       </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>Residential block one street south of Frat Row (113th); some weekend spillover, plus bar noise near the Broadway corner (The Heights, E's Bar around 112th–113th &amp; Broadway).</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
@@ -4809,6 +5634,16 @@
           <t>https://residential.columbia.edu/content/535-west-111th-street</t>
         </is>
       </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>Residential block; main noise vectors are the Broadway corner (The Heights bar at 111th &amp; Broadway) and some weekend spillover from the 113th–114th frat blocks two streets north.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
@@ -4867,6 +5702,16 @@
           <t>https://residential.columbia.edu/content/535-west-113th-street</t>
         </is>
       </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>On Columbia's Frat Row (W 113th–114th between Broadway and Amsterdam) amid active Greek houses (e.g. 534/536/540/548 W 114th, 556 W 113th). Expect weekend and late-night party noise — Columbia housing reviews flag this block as 'loud at night.'</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
@@ -4925,6 +5770,16 @@
           <t>https://residential.columbia.edu/content/536-west-113th-street</t>
         </is>
       </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>On Columbia's Frat Row (W 113th–114th between Broadway and Amsterdam) amid active Greek houses (e.g. 534/536/540/548 W 114th, 556 W 113th). Expect weekend and late-night party noise — Columbia housing reviews flag this block as 'loud at night.'</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
@@ -4983,6 +5838,16 @@
           <t>https://residential.columbia.edu/content/539-west-112th-street</t>
         </is>
       </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>Residential block one street south of Frat Row (113th); some weekend spillover, plus bar noise near the Broadway corner (The Heights, E's Bar around 112th–113th &amp; Broadway).</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
@@ -5041,6 +5906,16 @@
           <t>https://residential.columbia.edu/content/540-west-112th-street</t>
         </is>
       </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>Residential block one street south of Frat Row (113th); some weekend spillover, plus bar noise near the Broadway corner (The Heights, E's Bar around 112th–113th &amp; Broadway).</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
@@ -5099,6 +5974,16 @@
           <t>https://residential.columbia.edu/content/540-west-113th-street</t>
         </is>
       </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>On Columbia's Frat Row (W 113th–114th between Broadway and Amsterdam) amid active Greek houses (e.g. 534/536/540/548 W 114th, 556 W 113th). Expect weekend and late-night party noise — Columbia housing reviews flag this block as 'loud at night.'</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
@@ -5157,6 +6042,16 @@
           <t>https://residential.columbia.edu/content/540-west-122nd-street</t>
         </is>
       </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>Quiet faculty-housing side street between Amsterdam and Broadway, north of the main campus; little nightlife or through-traffic — main sound is daytime campus/sidewalk activity.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
@@ -5215,6 +6110,16 @@
           <t>https://residential.columbia.edu/content/541-west-113th-street</t>
         </is>
       </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>On Columbia's Frat Row (W 113th–114th between Broadway and Amsterdam) amid active Greek houses (e.g. 534/536/540/548 W 114th, 556 W 113th). Expect weekend and late-night party noise — Columbia housing reviews flag this block as 'loud at night.'</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
@@ -5273,6 +6178,16 @@
           <t>https://residential.columbia.edu/content/542-west-113th-street</t>
         </is>
       </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>On Columbia's Frat Row (W 113th–114th between Broadway and Amsterdam) amid active Greek houses (e.g. 534/536/540/548 W 114th, 556 W 113th). Expect weekend and late-night party noise — Columbia housing reviews flag this block as 'loud at night.'</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
@@ -5331,6 +6246,16 @@
           <t>https://residential.columbia.edu/content/544-west-113th-street</t>
         </is>
       </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>On Columbia's Frat Row (W 113th–114th between Broadway and Amsterdam) amid active Greek houses (e.g. 534/536/540/548 W 114th, 556 W 113th). Expect weekend and late-night party noise — Columbia housing reviews flag this block as 'loud at night.'</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
@@ -5389,6 +6314,16 @@
           <t>https://residential.columbia.edu/content/544-west-114th-street</t>
         </is>
       </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>On Columbia's Frat Row (W 113th–114th between Broadway and Amsterdam) amid active Greek houses (e.g. 534/536/540/548 W 114th, 556 W 113th). Expect weekend and late-night party noise — Columbia housing reviews flag this block as 'loud at night.'</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
@@ -5447,6 +6382,16 @@
           <t>https://residential.columbia.edu/content/547-riverside-drive</t>
         </is>
       </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>Park/parkway-facing Riverside Drive — among the quietest CR locations; only modest Riverside Dr through-traffic.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
@@ -5505,6 +6450,16 @@
           <t>https://residential.columbia.edu/content/548-riverside-drive</t>
         </is>
       </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>Park/parkway-facing Riverside Drive — among the quietest CR locations; only modest Riverside Dr through-traffic.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
@@ -5563,6 +6518,16 @@
           <t>https://residential.columbia.edu/content/549-riverside-drive</t>
         </is>
       </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>Park/parkway-facing Riverside Drive — among the quietest CR locations; only modest Riverside Dr through-traffic.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
@@ -5621,6 +6586,16 @@
           <t>https://residential.columbia.edu/content/554-west-113th-street</t>
         </is>
       </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>On Columbia's Frat Row (W 113th–114th between Broadway and Amsterdam) amid active Greek houses (e.g. 534/536/540/548 W 114th, 556 W 113th). Expect weekend and late-night party noise — Columbia housing reviews flag this block as 'loud at night.'</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
@@ -5679,6 +6654,16 @@
           <t>https://residential.columbia.edu/content/558-west-113th-street</t>
         </is>
       </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>On Columbia's Frat Row (W 113th–114th between Broadway and Amsterdam) amid active Greek houses (e.g. 534/536/540/548 W 114th, 556 W 113th). Expect weekend and late-night party noise — Columbia housing reviews flag this block as 'loud at night.'</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
@@ -5737,6 +6722,16 @@
           <t>https://residential.columbia.edu/content/560-west-113th-street</t>
         </is>
       </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>On Columbia's Frat Row (W 113th–114th between Broadway and Amsterdam) amid active Greek houses (e.g. 534/536/540/548 W 114th, 556 W 113th). Expect weekend and late-night party noise — Columbia housing reviews flag this block as 'loud at night.'</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
@@ -5795,6 +6790,16 @@
           <t>https://residential.columbia.edu/content/601-west-112th-street</t>
         </is>
       </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>West-of-Broadway end of W 112th toward Riverside — quiet residential, away from the frat blocks.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
@@ -5853,6 +6858,16 @@
           <t>https://residential.columbia.edu/content/601-west-113th-street</t>
         </is>
       </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>Quiet, west-of-Broadway end of W 113th toward Riverside — away from the fraternity houses on the Broadway–Amsterdam stretch.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
@@ -5911,6 +6926,16 @@
           <t>https://residential.columbia.edu/content/604-west-115th-street</t>
         </is>
       </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>West-of-Broadway end of W 115th toward Riverside — quiet residential.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
@@ -5969,6 +6994,16 @@
           <t>https://residential.columbia.edu/content/608-west-113th-street</t>
         </is>
       </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>Quiet, west-of-Broadway end of W 113th toward Riverside — away from the fraternity houses on the Broadway–Amsterdam stretch.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="8" t="inlineStr">
@@ -6027,6 +7062,16 @@
           <t>https://residential.columbia.edu/content/608-west-114th-street</t>
         </is>
       </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>Quiet, west-of-Broadway end of W 114th toward Riverside — away from the fraternity houses on the Broadway–Amsterdam stretch.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
@@ -6085,6 +7130,16 @@
           <t>https://residential.columbia.edu/content/610-west-113th-street</t>
         </is>
       </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>Quiet, west-of-Broadway end of W 113th toward Riverside — away from the fraternity houses on the Broadway–Amsterdam stretch.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
@@ -6143,6 +7198,16 @@
           <t>https://residential.columbia.edu/content/610-west-114th-street</t>
         </is>
       </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>Quiet, west-of-Broadway end of W 114th toward Riverside — away from the fraternity houses on the Broadway–Amsterdam stretch.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
@@ -6201,6 +7266,16 @@
           <t>https://residential.columbia.edu/content/610-west-115th-street</t>
         </is>
       </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>West-of-Broadway end of W 115th toward Riverside — quiet residential.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="8" t="inlineStr">
@@ -6259,6 +7334,16 @@
           <t>https://residential.columbia.edu/content/610-west-116th-street</t>
         </is>
       </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>Quiet residential block west of Broadway toward Riverside; minimal nightlife or arterial traffic.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
@@ -6317,6 +7402,16 @@
           <t>https://residential.columbia.edu/content/612-west-114th-street</t>
         </is>
       </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>Quiet, west-of-Broadway end of W 114th toward Riverside — away from the fraternity houses on the Broadway–Amsterdam stretch.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="8" t="inlineStr">
@@ -6375,6 +7470,16 @@
           <t>https://residential.columbia.edu/content/614-west-113th-street</t>
         </is>
       </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>Quiet, west-of-Broadway end of W 113th toward Riverside — away from the fraternity houses on the Broadway–Amsterdam stretch.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
@@ -6433,6 +7538,16 @@
           <t>https://residential.columbia.edu/content/617-west-115th-street</t>
         </is>
       </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>West-of-Broadway end of W 115th toward Riverside — quiet residential.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="8" t="inlineStr">
@@ -6491,6 +7606,16 @@
           <t>https://residential.columbia.edu/content/629-west-115th-street</t>
         </is>
       </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>West-of-Broadway end of W 115th toward Riverside — quiet residential.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
@@ -6549,6 +7674,16 @@
       <c r="L101" s="8" t="inlineStr">
         <is>
           <t>https://residential.columbia.edu/content/74-west-108th-street</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>Residential block between Amsterdam and Columbus on the UWS/Morningside edge; ordinary city-street traffic, no major nightlife on the block.</t>
         </is>
       </c>
     </row>

</xml_diff>